<commit_message>
update: 21.shleeclay CV 다운로드 단일화(full CV → Lee_Seunghyeon_Clay_CV.pdf) + cv 작업 파일 정리
- Contact 섹션 CV 다운로드를 간략/전체 2종에서 전체 CV 1종으로 단순화
- cvFullUrl → /cv/Lee_Seunghyeon_Clay_CV.pdf, cvSimplifiedUrl 제거
- cv/ 작업 파일(v3~v6 docx/pdf, short, old/, pys_old/, refs/) 추가
- .gitignore: *.tmp 전역 무시 추가

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cv/국가rnd정보.xlsx
+++ b/cv/국가rnd정보.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr defaultThemeVersion="202300"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="19029"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shlee\OneDrive\바탕 화면\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\20.git_research\01.topics\21.shleeclay.github.io\cv\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{56C58434-9C70-4E42-B8ED-F0DA0BE2E6CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="29020" windowHeight="17500" xr2:uid="{C8B435FE-D930-4C5B-8F1C-A0D2F2D5F71E}"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="29025" windowHeight="17505"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="85">
   <si>
     <t>내역사업명</t>
   </si>
@@ -293,12 +292,51 @@
   <si>
     <t>2019-04-17 ~ 2022-12-31</t>
   </si>
+  <si>
+    <t>습지생태계 가치증진 기술개발</t>
+  </si>
+  <si>
+    <t>상명대학교 천안산학협력단</t>
+  </si>
+  <si>
+    <t>탄소축적 묵논습지 조성 복원 관리기술</t>
+  </si>
+  <si>
+    <t>Creation Restoration and Management Technology of Carbon Accumulated Abandoned Paddy Wetland</t>
+  </si>
+  <si>
+    <t>충청남도  천안시</t>
+  </si>
+  <si>
+    <t>KE002322</t>
+  </si>
+  <si>
+    <t>2022-04-01 ~ 2026-12-31</t>
+  </si>
+  <si>
+    <t>2026-01-01 ~ 2026-12-31</t>
+  </si>
+  <si>
+    <r>
+      <t>작성대상과제가 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Noto Sans KR"/>
+        <family val="2"/>
+        <charset val="129"/>
+      </rPr>
+      <t>아닙니다.</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -382,6 +420,34 @@
       <color rgb="FFFF0000"/>
       <name val="Noto Sans KR"/>
       <family val="3"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Noto Sans KR"/>
+      <family val="2"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF962AF5"/>
+      <name val="Noto Sans KR"/>
+      <family val="2"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF6900"/>
+      <name val="Noto Sans KR"/>
+      <family val="2"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Noto Sans KR"/>
+      <family val="2"/>
       <charset val="129"/>
     </font>
   </fonts>
@@ -399,12 +465,27 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFDDDDDD"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFDDDDDD"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFDDDDDD"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFDDDDDD"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -413,7 +494,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -443,6 +524,18 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -777,11 +870,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3B27833-918D-4D6A-AAF5-6DF236D6AB43}">
-  <dimension ref="A1:I18"/>
-  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:J18"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:9" ht="74" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:10" ht="78.75" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -809,8 +902,11 @@
       <c r="I1" s="2" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" ht="55.5" x14ac:dyDescent="0.45">
+      <c r="J1" s="10" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="59.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -838,8 +934,11 @@
       <c r="I2" s="2" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" ht="111" x14ac:dyDescent="0.45">
+      <c r="J2" s="10" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="117.75" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
@@ -867,8 +966,11 @@
       <c r="I3" s="2" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" ht="259" x14ac:dyDescent="0.45">
+      <c r="J3" s="10" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="273.75" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
@@ -896,8 +998,11 @@
       <c r="I4" s="2" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="5" spans="1:9" ht="55.5" x14ac:dyDescent="0.45">
+      <c r="J4" s="10" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="59.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
@@ -925,8 +1030,11 @@
       <c r="I5" s="2" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="6" spans="1:9" ht="55.5" x14ac:dyDescent="0.45">
+      <c r="J5" s="10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="59.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>10</v>
       </c>
@@ -954,8 +1062,11 @@
       <c r="I6" s="2" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="7" spans="1:9" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="J6" s="10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="20.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>11</v>
       </c>
@@ -983,8 +1094,11 @@
       <c r="I7" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="8" spans="1:9" ht="37" x14ac:dyDescent="0.45">
+      <c r="J7" s="10" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="39.75" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>13</v>
       </c>
@@ -1012,8 +1126,11 @@
       <c r="I8" s="2" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="9" spans="1:9" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="J8" s="10" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="20.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>15</v>
       </c>
@@ -1041,8 +1158,11 @@
       <c r="I9" s="2" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="10" spans="1:9" ht="23" x14ac:dyDescent="0.45">
+      <c r="J9" s="10" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="20.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>17</v>
       </c>
@@ -1070,8 +1190,11 @@
       <c r="I10" s="3" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="11" spans="1:9" ht="37" x14ac:dyDescent="0.45">
+      <c r="J10" s="11" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="39.75" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>19</v>
       </c>
@@ -1099,8 +1222,11 @@
       <c r="I11" s="2" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="12" spans="1:9" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="J11" s="10" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="20.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>21</v>
       </c>
@@ -1128,8 +1254,11 @@
       <c r="I12" s="4">
         <v>1485018680</v>
       </c>
-    </row>
-    <row r="13" spans="1:9" ht="37" x14ac:dyDescent="0.45">
+      <c r="J12" s="12">
+        <v>2050001587</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="39.75" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>22</v>
       </c>
@@ -1157,8 +1286,11 @@
       <c r="I13" s="2" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="14" spans="1:9" ht="74" x14ac:dyDescent="0.45">
+      <c r="J13" s="10" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="59.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>24</v>
       </c>
@@ -1186,8 +1318,11 @@
       <c r="I14" s="2" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="15" spans="1:9" ht="74" x14ac:dyDescent="0.45">
+      <c r="J14" s="10" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="59.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>26</v>
       </c>
@@ -1215,8 +1350,11 @@
       <c r="I15" s="2" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="16" spans="1:9" ht="37" x14ac:dyDescent="0.45">
+      <c r="J15" s="10" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="39.75" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>28</v>
       </c>
@@ -1238,8 +1376,11 @@
       <c r="I16" s="2" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="17" spans="1:9" ht="55.5" x14ac:dyDescent="0.45">
+      <c r="J16" s="10" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="59.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>30</v>
       </c>
@@ -1261,8 +1402,11 @@
       <c r="I17" s="2" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="18" spans="1:9" ht="23" x14ac:dyDescent="0.45">
+      <c r="J17" s="10" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="19.5" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>32</v>
       </c>
@@ -1289,6 +1433,9 @@
       </c>
       <c r="I18" s="6">
         <v>735</v>
+      </c>
+      <c r="J18" s="13">
+        <v>546.66999999999996</v>
       </c>
     </row>
   </sheetData>

</xml_diff>